<commit_message>
Update Job Scout search backends and diagnostics
</commit_message>
<xml_diff>
--- a/output/job-tracker.xlsx
+++ b/output/job-tracker.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Tracker'!$A$1:$N$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Scout'!$A$1:$W$848</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Scout'!$A$1:$W$907</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -4534,7 +4534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W848"/>
+  <dimension ref="A1:W907"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5015,7 +5015,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="U5" s="719" t="n"/>
+      <c r="U5" s="719" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="V5" s="719" t="inlineStr">
         <is>
           <t>file:///C:/Users/DCALL/Desktop/gecko/output/resumes/Dave-Call%2BIncorta%2Bf813a666-81a8-45be-ba2f-9f447edce30e.docx</t>
@@ -68830,8 +68834,4447 @@
       <c r="V848" s="719" t="n"/>
       <c r="W848" s="719" t="n"/>
     </row>
+    <row r="849">
+      <c r="A849" s="719" t="n">
+        <v>848</v>
+      </c>
+      <c r="B849" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C849" s="719" t="inlineStr">
+        <is>
+          <t>Five Star Franchising</t>
+        </is>
+      </c>
+      <c r="D849" s="719" t="inlineStr">
+        <is>
+          <t>Director of Performance Marketing</t>
+        </is>
+      </c>
+      <c r="E849" s="722" t="n">
+        <v>70</v>
+      </c>
+      <c r="F849" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G849" s="719" t="inlineStr">
+        <is>
+          <t>Near Match</t>
+        </is>
+      </c>
+      <c r="H849" s="719" t="inlineStr">
+        <is>
+          <t>Springville, UT</t>
+        </is>
+      </c>
+      <c r="I849" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J849" s="719" t="n"/>
+      <c r="K849" s="719" t="n"/>
+      <c r="L849" s="720" t="n">
+        <v>46283</v>
+      </c>
+      <c r="M849" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N849" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O849" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P849" s="719" t="n"/>
+      <c r="Q849" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-6607435749910257112?p=1&amp;pos=3&amp;rgn=45&amp;cid=19881&amp;ckey=Paid+Search+Manager&amp;jobAge=112&amp;brelb=100&amp;scr=71.81189&amp;bscr=71.81189&amp;aq=5557669938633344924&amp;elckey=2496484699213495798</t>
+        </is>
+      </c>
+      <c r="R849" s="719" t="n"/>
+      <c r="S849" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T849" s="719" t="n"/>
+      <c r="U849" s="719" t="n"/>
+      <c r="V849" s="719" t="n"/>
+      <c r="W849" s="719" t="n"/>
+    </row>
+    <row r="850">
+      <c r="A850" s="719" t="n">
+        <v>849</v>
+      </c>
+      <c r="B850" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C850" s="719" t="inlineStr">
+        <is>
+          <t>MoneyLion</t>
+        </is>
+      </c>
+      <c r="D850" s="719" t="inlineStr">
+        <is>
+          <t>Senior Paid Search Specialist</t>
+        </is>
+      </c>
+      <c r="E850" s="722" t="n">
+        <v>59</v>
+      </c>
+      <c r="F850" s="723" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G850" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H850" s="719" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="I850" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J850" s="719" t="inlineStr">
+        <is>
+          <t>full-time</t>
+        </is>
+      </c>
+      <c r="K850" s="719" t="inlineStr">
+        <is>
+          <t>$100k - $115k</t>
+        </is>
+      </c>
+      <c r="L850" s="720" t="n">
+        <v>46276</v>
+      </c>
+      <c r="M850" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N850" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O850" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P850" s="719" t="n"/>
+      <c r="Q850" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/desc/-3578475564271799010?ckey=Paid+Search+Specialist&amp;rgn=55157&amp;pos=9&amp;groupId=41016&amp;elckey=-6101355134584310867&amp;p=1&amp;aq=-6854990064588241940&amp;cid=19881&amp;jobAge=280&amp;brelb=100&amp;bscr=1669.6665&amp;scr=1669.6665</t>
+        </is>
+      </c>
+      <c r="R850" s="719" t="n"/>
+      <c r="S850" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T850" s="719" t="n"/>
+      <c r="U850" s="719" t="n"/>
+      <c r="V850" s="719" t="n"/>
+      <c r="W850" s="719" t="n"/>
+    </row>
+    <row r="851">
+      <c r="A851" s="719" t="n">
+        <v>850</v>
+      </c>
+      <c r="B851" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C851" s="719" t="inlineStr">
+        <is>
+          <t>Unavailable</t>
+        </is>
+      </c>
+      <c r="D851" s="719" t="inlineStr">
+        <is>
+          <t>Coordinator, Paid Search</t>
+        </is>
+      </c>
+      <c r="E851" s="722" t="n">
+        <v>44</v>
+      </c>
+      <c r="F851" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G851" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H851" s="719" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="I851" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J851" s="719" t="n"/>
+      <c r="K851" s="719" t="inlineStr">
+        <is>
+          <t>$50k</t>
+        </is>
+      </c>
+      <c r="L851" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M851" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N851" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O851" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P851" s="719" t="n"/>
+      <c r="Q851" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-4821031450085058660?p=1&amp;pos=16&amp;rgn=55157&amp;cid=19881&amp;ckey=Paid+Search+Specialist&amp;jobAge=40&amp;brelb=100&amp;scr=1057.3561&amp;bscr=1057.3561&amp;aq=-6854990064588241940&amp;elckey=-6101355134584310867</t>
+        </is>
+      </c>
+      <c r="R851" s="719" t="n"/>
+      <c r="S851" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T851" s="719" t="n"/>
+      <c r="U851" s="719" t="n"/>
+      <c r="V851" s="719" t="n"/>
+      <c r="W851" s="719" t="n"/>
+    </row>
+    <row r="852">
+      <c r="A852" s="719" t="n">
+        <v>851</v>
+      </c>
+      <c r="B852" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C852" s="719" t="inlineStr">
+        <is>
+          <t>Directive Consulting</t>
+        </is>
+      </c>
+      <c r="D852" s="719" t="inlineStr">
+        <is>
+          <t>PPC Manager (Remote US)</t>
+        </is>
+      </c>
+      <c r="E852" s="722" t="n">
+        <v>66</v>
+      </c>
+      <c r="F852" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G852" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H852" s="719" t="inlineStr">
+        <is>
+          <t>Kansas City, MO</t>
+        </is>
+      </c>
+      <c r="I852" s="719" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="J852" s="719" t="n"/>
+      <c r="K852" s="719" t="inlineStr">
+        <is>
+          <t>$70k - $95k</t>
+        </is>
+      </c>
+      <c r="L852" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M852" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N852" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O852" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P852" s="719" t="n"/>
+      <c r="Q852" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-6466330632279687363?p=1&amp;pos=10&amp;rgn=55157&amp;cid=19881&amp;ckey=PPC+Manager&amp;jobAge=88&amp;brelb=100&amp;scr=161.4026&amp;bscr=161.4026&amp;aq=2743865504884634649&amp;elckey=-4582280812807247181</t>
+        </is>
+      </c>
+      <c r="R852" s="719" t="n"/>
+      <c r="S852" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T852" s="719" t="n"/>
+      <c r="U852" s="719" t="n"/>
+      <c r="V852" s="719" t="n"/>
+      <c r="W852" s="719" t="n"/>
+    </row>
+    <row r="853">
+      <c r="A853" s="719" t="n">
+        <v>852</v>
+      </c>
+      <c r="B853" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C853" s="719" t="inlineStr">
+        <is>
+          <t>Audacy</t>
+        </is>
+      </c>
+      <c r="D853" s="719" t="inlineStr">
+        <is>
+          <t>Search Engine Marketing (SEM) Account Manager</t>
+        </is>
+      </c>
+      <c r="E853" s="722" t="n">
+        <v>45</v>
+      </c>
+      <c r="F853" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G853" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H853" s="719" t="inlineStr">
+        <is>
+          <t>Baltimore, MD</t>
+        </is>
+      </c>
+      <c r="I853" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J853" s="719" t="n"/>
+      <c r="K853" s="719" t="inlineStr">
+        <is>
+          <t>$55k - $65k</t>
+        </is>
+      </c>
+      <c r="L853" s="720" t="n">
+        <v>46283</v>
+      </c>
+      <c r="M853" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N853" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O853" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P853" s="719" t="n"/>
+      <c r="Q853" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-362832477277684754?p=1&amp;pos=2&amp;rgn=55157&amp;cid=19881&amp;ckey=SEM+Manager&amp;jobAge=110&amp;brelb=100&amp;scr=716.45123&amp;bscr=716.45123&amp;aq=1505378311137433824&amp;elckey=-4304702802211614107</t>
+        </is>
+      </c>
+      <c r="R853" s="719" t="n"/>
+      <c r="S853" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T853" s="719" t="n"/>
+      <c r="U853" s="719" t="n"/>
+      <c r="V853" s="719" t="n"/>
+      <c r="W853" s="719" t="n"/>
+    </row>
+    <row r="854">
+      <c r="A854" s="719" t="n">
+        <v>853</v>
+      </c>
+      <c r="B854" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C854" s="719" t="inlineStr">
+        <is>
+          <t>Doordash</t>
+        </is>
+      </c>
+      <c r="D854" s="719" t="inlineStr">
+        <is>
+          <t>Associate Manager, Consumer Integrated Marketing - New Verticals Habituation</t>
+        </is>
+      </c>
+      <c r="E854" s="722" t="n">
+        <v>56</v>
+      </c>
+      <c r="F854" s="723" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G854" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H854" s="719" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="I854" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J854" s="719" t="n"/>
+      <c r="K854" s="719" t="inlineStr">
+        <is>
+          <t>$108.8k - $160k</t>
+        </is>
+      </c>
+      <c r="L854" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M854" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N854" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O854" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P854" s="719" t="n"/>
+      <c r="Q854" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/4485297588300984488?p=1&amp;pos=19&amp;rgn=55157&amp;cid=19881&amp;ckey=SEM+Manager&amp;jobAge=64&amp;brelb=100&amp;scr=184.7804&amp;bscr=184.7804&amp;aq=1505378311137433824&amp;elckey=-4304702802211614107</t>
+        </is>
+      </c>
+      <c r="R854" s="719" t="n"/>
+      <c r="S854" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T854" s="719" t="n"/>
+      <c r="U854" s="719" t="n"/>
+      <c r="V854" s="719" t="n"/>
+      <c r="W854" s="719" t="n"/>
+    </row>
+    <row r="855">
+      <c r="A855" s="719" t="n">
+        <v>854</v>
+      </c>
+      <c r="B855" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C855" s="719" t="inlineStr">
+        <is>
+          <t>Zimmer Communications</t>
+        </is>
+      </c>
+      <c r="D855" s="719" t="inlineStr">
+        <is>
+          <t>Digital Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E855" s="722" t="n">
+        <v>56</v>
+      </c>
+      <c r="F855" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G855" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H855" s="719" t="inlineStr">
+        <is>
+          <t>Columbia, MO</t>
+        </is>
+      </c>
+      <c r="I855" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J855" s="719" t="n"/>
+      <c r="K855" s="719" t="n"/>
+      <c r="L855" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M855" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N855" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O855" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P855" s="719" t="n"/>
+      <c r="Q855" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-3476186282926399677?p=1&amp;pos=19&amp;rgn=55157&amp;cid=19881&amp;ckey=Digital+Marketing+Manager&amp;jobAge=88&amp;brelb=10&amp;scr=185.00194&amp;bscr=185.00194&amp;aq=8330494891823432483&amp;elckey=-2444203368392194727</t>
+        </is>
+      </c>
+      <c r="R855" s="719" t="n"/>
+      <c r="S855" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T855" s="719" t="n"/>
+      <c r="U855" s="719" t="n"/>
+      <c r="V855" s="719" t="n"/>
+      <c r="W855" s="719" t="n"/>
+    </row>
+    <row r="856">
+      <c r="A856" s="719" t="n">
+        <v>855</v>
+      </c>
+      <c r="B856" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C856" s="719" t="inlineStr">
+        <is>
+          <t>Socket.dev</t>
+        </is>
+      </c>
+      <c r="D856" s="719" t="inlineStr">
+        <is>
+          <t>Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E856" s="722" t="n">
+        <v>43</v>
+      </c>
+      <c r="F856" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G856" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H856" s="719" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="I856" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J856" s="719" t="n"/>
+      <c r="K856" s="719" t="n"/>
+      <c r="L856" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M856" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N856" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O856" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P856" s="719" t="n"/>
+      <c r="Q856" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/3962202025831574032?p=1&amp;pos=6&amp;rgn=45&amp;cid=19881&amp;ckey=Search+Marketing+Manager&amp;jobAge=64&amp;brelb=100&amp;scr=181.40236&amp;bscr=181.40236&amp;aq=-1548421499840547201&amp;elckey=-8967727484152184132</t>
+        </is>
+      </c>
+      <c r="R856" s="719" t="n"/>
+      <c r="S856" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T856" s="719" t="n"/>
+      <c r="U856" s="719" t="n"/>
+      <c r="V856" s="719" t="n"/>
+      <c r="W856" s="719" t="n"/>
+    </row>
+    <row r="857">
+      <c r="A857" s="719" t="n">
+        <v>856</v>
+      </c>
+      <c r="B857" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C857" s="719" t="inlineStr">
+        <is>
+          <t>Roku, Inc.</t>
+        </is>
+      </c>
+      <c r="D857" s="719" t="inlineStr">
+        <is>
+          <t>Paid Search Manager</t>
+        </is>
+      </c>
+      <c r="E857" s="722" t="n">
+        <v>61</v>
+      </c>
+      <c r="F857" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G857" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H857" s="719" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="I857" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J857" s="719" t="n"/>
+      <c r="K857" s="719" t="inlineStr">
+        <is>
+          <t>$108k - $121k</t>
+        </is>
+      </c>
+      <c r="L857" s="720" t="n">
+        <v>46282</v>
+      </c>
+      <c r="M857" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N857" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O857" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P857" s="719" t="n"/>
+      <c r="Q857" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/8948860322612986060?p=1&amp;pos=20&amp;rgn=55157&amp;cid=19881&amp;ckey=Search+Marketing+Manager&amp;jobAge=136&amp;brelb=100&amp;scr=894.0899&amp;bscr=894.0899&amp;aq=-2163660769833457005&amp;elckey=-1151053109316742606</t>
+        </is>
+      </c>
+      <c r="R857" s="719" t="n"/>
+      <c r="S857" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T857" s="719" t="n"/>
+      <c r="U857" s="719" t="n"/>
+      <c r="V857" s="719" t="n"/>
+      <c r="W857" s="719" t="n"/>
+    </row>
+    <row r="858">
+      <c r="A858" s="719" t="n">
+        <v>857</v>
+      </c>
+      <c r="B858" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C858" s="719" t="inlineStr">
+        <is>
+          <t>Mister Car Wash</t>
+        </is>
+      </c>
+      <c r="D858" s="719" t="inlineStr">
+        <is>
+          <t>Head of Growth Marketing</t>
+        </is>
+      </c>
+      <c r="E858" s="722" t="n">
+        <v>61</v>
+      </c>
+      <c r="F858" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G858" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H858" s="719" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="I858" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J858" s="719" t="n"/>
+      <c r="K858" s="719" t="n"/>
+      <c r="L858" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M858" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N858" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O858" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P858" s="719" t="n"/>
+      <c r="Q858" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/4185722973533811702?p=1&amp;pos=18&amp;rgn=45&amp;cid=19881&amp;ckey=Marketing+Analytics+Manager&amp;jobAge=40&amp;brelb=100&amp;scr=200.93472&amp;bscr=200.93472&amp;aq=6699460534411435160&amp;elckey=4840406746592066267</t>
+        </is>
+      </c>
+      <c r="R858" s="719" t="n"/>
+      <c r="S858" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T858" s="719" t="n"/>
+      <c r="U858" s="719" t="n"/>
+      <c r="V858" s="719" t="n"/>
+      <c r="W858" s="719" t="n"/>
+    </row>
+    <row r="859">
+      <c r="A859" s="719" t="n">
+        <v>858</v>
+      </c>
+      <c r="B859" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C859" s="719" t="inlineStr">
+        <is>
+          <t>IXL</t>
+        </is>
+      </c>
+      <c r="D859" s="719" t="inlineStr">
+        <is>
+          <t>Digital Marketing Analyst</t>
+        </is>
+      </c>
+      <c r="E859" s="722" t="n">
+        <v>48</v>
+      </c>
+      <c r="F859" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G859" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H859" s="719" t="inlineStr">
+        <is>
+          <t>San Mateo, CA</t>
+        </is>
+      </c>
+      <c r="I859" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J859" s="719" t="n"/>
+      <c r="K859" s="719" t="inlineStr">
+        <is>
+          <t>$70.3k - $75k</t>
+        </is>
+      </c>
+      <c r="L859" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M859" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N859" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O859" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P859" s="719" t="n"/>
+      <c r="Q859" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/63120824566342626?p=1&amp;pos=12&amp;rgn=55157&amp;cid=19881&amp;ckey=Digital+Marketing+Analyst&amp;jobAge=40&amp;brelb=100&amp;scr=1764.9364&amp;bscr=1764.9364&amp;aq=-2656194179588722569&amp;elckey=-8685117671900227655</t>
+        </is>
+      </c>
+      <c r="R859" s="719" t="n"/>
+      <c r="S859" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T859" s="719" t="n"/>
+      <c r="U859" s="719" t="n"/>
+      <c r="V859" s="719" t="n"/>
+      <c r="W859" s="719" t="n"/>
+    </row>
+    <row r="860">
+      <c r="A860" s="719" t="n">
+        <v>859</v>
+      </c>
+      <c r="B860" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C860" s="719" t="inlineStr">
+        <is>
+          <t>CMI Media and Compas</t>
+        </is>
+      </c>
+      <c r="D860" s="719" t="inlineStr">
+        <is>
+          <t>Senior Analyst, Digital Marketing Analytics</t>
+        </is>
+      </c>
+      <c r="E860" s="722" t="n">
+        <v>58</v>
+      </c>
+      <c r="F860" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G860" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H860" s="719" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA</t>
+        </is>
+      </c>
+      <c r="I860" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J860" s="719" t="n"/>
+      <c r="K860" s="719" t="inlineStr">
+        <is>
+          <t>$50k - $90k</t>
+        </is>
+      </c>
+      <c r="L860" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M860" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N860" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O860" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P860" s="719" t="n"/>
+      <c r="Q860" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/2076542528262505103?p=1&amp;pos=20&amp;rgn=55157&amp;cid=19881&amp;ckey=Digital+Marketing+Analyst&amp;jobAge=88&amp;brelb=100&amp;scr=374.0575&amp;bscr=374.0575&amp;aq=-2656194179588722569&amp;elckey=-8685117671900227655</t>
+        </is>
+      </c>
+      <c r="R860" s="719" t="n"/>
+      <c r="S860" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T860" s="719" t="n"/>
+      <c r="U860" s="719" t="n"/>
+      <c r="V860" s="719" t="n"/>
+      <c r="W860" s="719" t="n"/>
+    </row>
+    <row r="861">
+      <c r="A861" s="719" t="n">
+        <v>860</v>
+      </c>
+      <c r="B861" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C861" s="719" t="inlineStr">
+        <is>
+          <t>Priceline.com</t>
+        </is>
+      </c>
+      <c r="D861" s="719" t="inlineStr">
+        <is>
+          <t>App Growth Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E861" s="722" t="n">
+        <v>67</v>
+      </c>
+      <c r="F861" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G861" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H861" s="719" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="I861" s="719" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="J861" s="719" t="n"/>
+      <c r="K861" s="719" t="n"/>
+      <c r="L861" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M861" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N861" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O861" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P861" s="719" t="n"/>
+      <c r="Q861" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-4929761423494631778?p=1&amp;pos=5&amp;rgn=55157&amp;cid=19881&amp;ckey=Growth+Marketing+Manager&amp;jobAge=40&amp;brelb=100&amp;scr=666.31226&amp;bscr=666.31226&amp;aq=1924841946078193672&amp;elckey=-3752150848771295917</t>
+        </is>
+      </c>
+      <c r="R861" s="719" t="n"/>
+      <c r="S861" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T861" s="719" t="n"/>
+      <c r="U861" s="719" t="n"/>
+      <c r="V861" s="719" t="n"/>
+      <c r="W861" s="719" t="n"/>
+    </row>
+    <row r="862">
+      <c r="A862" s="719" t="n">
+        <v>861</v>
+      </c>
+      <c r="B862" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C862" s="719" t="inlineStr">
+        <is>
+          <t>Brex</t>
+        </is>
+      </c>
+      <c r="D862" s="719" t="inlineStr">
+        <is>
+          <t>Senior Growth Marketing Manager, Paid Social</t>
+        </is>
+      </c>
+      <c r="E862" s="722" t="n">
+        <v>66</v>
+      </c>
+      <c r="F862" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G862" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H862" s="719" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
+      <c r="I862" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J862" s="719" t="n"/>
+      <c r="K862" s="719" t="inlineStr">
+        <is>
+          <t>$131.08k - $163.85k</t>
+        </is>
+      </c>
+      <c r="L862" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M862" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N862" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O862" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P862" s="719" t="n"/>
+      <c r="Q862" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/3684436537288614143?p=1&amp;pos=8&amp;rgn=55157&amp;cid=19881&amp;ckey=Growth+Marketing+Manager&amp;jobAge=61&amp;brelb=100&amp;scr=665.7932&amp;bscr=665.7932&amp;aq=1924841946078193672&amp;elckey=-3752150848771295917</t>
+        </is>
+      </c>
+      <c r="R862" s="719" t="n"/>
+      <c r="S862" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T862" s="719" t="n"/>
+      <c r="U862" s="719" t="n"/>
+      <c r="V862" s="719" t="n"/>
+      <c r="W862" s="719" t="n"/>
+    </row>
+    <row r="863">
+      <c r="A863" s="719" t="n">
+        <v>862</v>
+      </c>
+      <c r="B863" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C863" s="719" t="inlineStr">
+        <is>
+          <t>OSavul, Inc.</t>
+        </is>
+      </c>
+      <c r="D863" s="719" t="inlineStr">
+        <is>
+          <t>Demand Generation Manager</t>
+        </is>
+      </c>
+      <c r="E863" s="722" t="n">
+        <v>66</v>
+      </c>
+      <c r="F863" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G863" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H863" s="719" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I863" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J863" s="719" t="n"/>
+      <c r="K863" s="719" t="n"/>
+      <c r="L863" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M863" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N863" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O863" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P863" s="719" t="n"/>
+      <c r="Q863" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-394938773360978355?p=1&amp;pos=20&amp;rgn=55157&amp;cid=19881&amp;ckey=Demand+Generation+Manager&amp;jobAge=16&amp;brelb=10&amp;scr=161.50073&amp;bscr=161.50073&amp;aq=3135917889178899316&amp;elckey=5432738477877767859</t>
+        </is>
+      </c>
+      <c r="R863" s="719" t="n"/>
+      <c r="S863" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T863" s="719" t="n"/>
+      <c r="U863" s="719" t="n"/>
+      <c r="V863" s="719" t="n"/>
+      <c r="W863" s="719" t="n"/>
+    </row>
+    <row r="864">
+      <c r="A864" s="719" t="n">
+        <v>863</v>
+      </c>
+      <c r="B864" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C864" s="719" t="inlineStr">
+        <is>
+          <t>Directive Consulting</t>
+        </is>
+      </c>
+      <c r="D864" s="719" t="inlineStr">
+        <is>
+          <t>Senior Account Strategist, Paid Media (Remote US)</t>
+        </is>
+      </c>
+      <c r="E864" s="722" t="n">
+        <v>43</v>
+      </c>
+      <c r="F864" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G864" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H864" s="719" t="inlineStr">
+        <is>
+          <t>Richmond, VA</t>
+        </is>
+      </c>
+      <c r="I864" s="719" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="J864" s="719" t="n"/>
+      <c r="K864" s="719" t="inlineStr">
+        <is>
+          <t>$90k - $110k</t>
+        </is>
+      </c>
+      <c r="L864" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M864" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N864" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O864" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P864" s="719" t="n"/>
+      <c r="Q864" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/6365963937850806933?p=1&amp;pos=9&amp;rgn=55157&amp;cid=19881&amp;ckey=Senior+Paid+Search+Strategist&amp;jobAge=88&amp;brelb=100&amp;scr=5648.84&amp;bscr=5648.84&amp;aq=4816781853536242611&amp;elckey=8918642023499669742</t>
+        </is>
+      </c>
+      <c r="R864" s="719" t="n"/>
+      <c r="S864" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T864" s="719" t="n"/>
+      <c r="U864" s="719" t="n"/>
+      <c r="V864" s="719" t="n"/>
+      <c r="W864" s="719" t="n"/>
+    </row>
+    <row r="865">
+      <c r="A865" s="719" t="n">
+        <v>864</v>
+      </c>
+      <c r="B865" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C865" s="719" t="inlineStr">
+        <is>
+          <t>Tech9</t>
+        </is>
+      </c>
+      <c r="D865" s="719" t="inlineStr">
+        <is>
+          <t>Paid Search Manager</t>
+        </is>
+      </c>
+      <c r="E865" s="722" t="n">
+        <v>73</v>
+      </c>
+      <c r="F865" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G865" s="719" t="inlineStr">
+        <is>
+          <t>Near Match</t>
+        </is>
+      </c>
+      <c r="H865" s="719" t="inlineStr">
+        <is>
+          <t>Vineyard, UT</t>
+        </is>
+      </c>
+      <c r="I865" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J865" s="719" t="n"/>
+      <c r="K865" s="719" t="n"/>
+      <c r="L865" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M865" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N865" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O865" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P865" s="719" t="n"/>
+      <c r="Q865" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-1936297981840618732?p=1&amp;pos=1&amp;rgn=45&amp;cid=19881&amp;ckey=Paid+Search+Manager&amp;jobAge=66&amp;brelb=10&amp;scr=205.15237&amp;bscr=205.15237&amp;aq=-1169608878158539505&amp;elckey=-1481818911242664502</t>
+        </is>
+      </c>
+      <c r="R865" s="719" t="n"/>
+      <c r="S865" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T865" s="719" t="n"/>
+      <c r="U865" s="719" t="n"/>
+      <c r="V865" s="719" t="n"/>
+      <c r="W865" s="719" t="n"/>
+    </row>
+    <row r="866">
+      <c r="A866" s="719" t="n">
+        <v>865</v>
+      </c>
+      <c r="B866" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C866" s="719" t="inlineStr">
+        <is>
+          <t>Brady</t>
+        </is>
+      </c>
+      <c r="D866" s="719" t="inlineStr">
+        <is>
+          <t>Performance Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E866" s="722" t="n">
+        <v>71</v>
+      </c>
+      <c r="F866" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G866" s="719" t="inlineStr">
+        <is>
+          <t>Near Match</t>
+        </is>
+      </c>
+      <c r="H866" s="719" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="I866" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J866" s="719" t="n"/>
+      <c r="K866" s="719" t="n"/>
+      <c r="L866" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M866" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N866" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O866" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P866" s="719" t="n"/>
+      <c r="Q866" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/498601059327496963?p=1&amp;pos=2&amp;rgn=45&amp;cid=19881&amp;ckey=Paid+Search+Manager&amp;jobAge=90&amp;brelb=10&amp;scr=88.58706&amp;bscr=88.58706&amp;aq=-1169608878158539505&amp;elckey=-1481818911242664502</t>
+        </is>
+      </c>
+      <c r="R866" s="719" t="n"/>
+      <c r="S866" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T866" s="719" t="n"/>
+      <c r="U866" s="719" t="n"/>
+      <c r="V866" s="719" t="n"/>
+      <c r="W866" s="719" t="n"/>
+    </row>
+    <row r="867">
+      <c r="A867" s="719" t="n">
+        <v>866</v>
+      </c>
+      <c r="B867" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C867" s="719" t="inlineStr">
+        <is>
+          <t>ClearCompanies</t>
+        </is>
+      </c>
+      <c r="D867" s="719" t="inlineStr">
+        <is>
+          <t>DIgital Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E867" s="722" t="n">
+        <v>72</v>
+      </c>
+      <c r="F867" s="723" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G867" s="719" t="inlineStr">
+        <is>
+          <t>Near Match</t>
+        </is>
+      </c>
+      <c r="H867" s="719" t="inlineStr">
+        <is>
+          <t>Orem, UT</t>
+        </is>
+      </c>
+      <c r="I867" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J867" s="719" t="n"/>
+      <c r="K867" s="719" t="n"/>
+      <c r="L867" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M867" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N867" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O867" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P867" s="719" t="n"/>
+      <c r="Q867" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/2637774066161055811?p=1&amp;pos=11&amp;rgn=45&amp;cid=19881&amp;ckey=Paid+Search+Manager&amp;jobAge=66&amp;brelb=10&amp;scr=49.207413&amp;bscr=49.207413&amp;aq=-1169608878158539505&amp;elckey=-1481818911242664502</t>
+        </is>
+      </c>
+      <c r="R867" s="719" t="n"/>
+      <c r="S867" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T867" s="719" t="n"/>
+      <c r="U867" s="719" t="n"/>
+      <c r="V867" s="719" t="n"/>
+      <c r="W867" s="719" t="n"/>
+    </row>
+    <row r="868">
+      <c r="A868" s="719" t="n">
+        <v>867</v>
+      </c>
+      <c r="B868" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C868" s="719" t="inlineStr">
+        <is>
+          <t>Resolut Inc</t>
+        </is>
+      </c>
+      <c r="D868" s="719" t="inlineStr">
+        <is>
+          <t>Digital Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E868" s="722" t="n">
+        <v>71</v>
+      </c>
+      <c r="F868" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G868" s="719" t="inlineStr">
+        <is>
+          <t>Near Match</t>
+        </is>
+      </c>
+      <c r="H868" s="719" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="I868" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J868" s="719" t="n"/>
+      <c r="K868" s="719" t="n"/>
+      <c r="L868" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M868" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N868" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O868" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P868" s="719" t="n"/>
+      <c r="Q868" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/3807486199544679677?p=1&amp;pos=12&amp;rgn=45&amp;cid=19881&amp;ckey=Paid+Search+Manager&amp;jobAge=42&amp;brelb=10&amp;scr=49.207413&amp;bscr=49.207413&amp;aq=-1169608878158539505&amp;elckey=-1481818911242664502</t>
+        </is>
+      </c>
+      <c r="R868" s="719" t="n"/>
+      <c r="S868" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T868" s="719" t="n"/>
+      <c r="U868" s="719" t="n"/>
+      <c r="V868" s="719" t="n"/>
+      <c r="W868" s="719" t="n"/>
+    </row>
+    <row r="869">
+      <c r="A869" s="719" t="n">
+        <v>868</v>
+      </c>
+      <c r="B869" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C869" s="719" t="inlineStr">
+        <is>
+          <t>Socket.dev</t>
+        </is>
+      </c>
+      <c r="D869" s="719" t="inlineStr">
+        <is>
+          <t>Paid Search Manager</t>
+        </is>
+      </c>
+      <c r="E869" s="722" t="n">
+        <v>73</v>
+      </c>
+      <c r="F869" s="723" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G869" s="719" t="inlineStr">
+        <is>
+          <t>Near Match</t>
+        </is>
+      </c>
+      <c r="H869" s="719" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="I869" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J869" s="719" t="n"/>
+      <c r="K869" s="719" t="inlineStr">
+        <is>
+          <t>$85k - $95k</t>
+        </is>
+      </c>
+      <c r="L869" s="720" t="n">
+        <v>46282</v>
+      </c>
+      <c r="M869" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N869" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O869" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P869" s="719" t="n"/>
+      <c r="Q869" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-8833274305632955408?p=1&amp;pos=18&amp;rgn=55157&amp;cid=19881&amp;ckey=Paid+Search+Manager&amp;jobAge=138&amp;brelb=100&amp;scr=165.26001&amp;bscr=165.26001&amp;aq=-17202559000866049&amp;elckey=-2609051204955160592</t>
+        </is>
+      </c>
+      <c r="R869" s="719" t="n"/>
+      <c r="S869" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T869" s="719" t="n"/>
+      <c r="U869" s="719" t="n"/>
+      <c r="V869" s="719" t="n"/>
+      <c r="W869" s="719" t="n"/>
+    </row>
+    <row r="870">
+      <c r="A870" s="719" t="n">
+        <v>869</v>
+      </c>
+      <c r="B870" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C870" s="719" t="inlineStr">
+        <is>
+          <t>3 Little Birds Interactive</t>
+        </is>
+      </c>
+      <c r="D870" s="719" t="inlineStr">
+        <is>
+          <t>Paid Search Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E870" s="722" t="n">
+        <v>57</v>
+      </c>
+      <c r="F870" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G870" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H870" s="719" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I870" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J870" s="719" t="n"/>
+      <c r="K870" s="719" t="n"/>
+      <c r="L870" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M870" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N870" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O870" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P870" s="719" t="n"/>
+      <c r="Q870" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-9018681185510549445?p=1&amp;pos=19&amp;rgn=55157&amp;cid=19881&amp;ckey=Paid+Search+Manager&amp;jobAge=66&amp;brelb=100&amp;scr=160.85867&amp;bscr=160.85867&amp;aq=-17202559000866049&amp;elckey=-2609051204955160592</t>
+        </is>
+      </c>
+      <c r="R870" s="719" t="n"/>
+      <c r="S870" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T870" s="719" t="n"/>
+      <c r="U870" s="719" t="n"/>
+      <c r="V870" s="719" t="n"/>
+      <c r="W870" s="719" t="n"/>
+    </row>
+    <row r="871">
+      <c r="A871" s="719" t="n">
+        <v>870</v>
+      </c>
+      <c r="B871" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C871" s="719" t="inlineStr">
+        <is>
+          <t>Rithum</t>
+        </is>
+      </c>
+      <c r="D871" s="719" t="inlineStr">
+        <is>
+          <t>Remote Advertising Paid Search Manager - Ecommerce</t>
+        </is>
+      </c>
+      <c r="E871" s="722" t="n">
+        <v>72</v>
+      </c>
+      <c r="F871" s="723" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G871" s="719" t="inlineStr">
+        <is>
+          <t>Near Match</t>
+        </is>
+      </c>
+      <c r="H871" s="719" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="I871" s="719" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="J871" s="719" t="inlineStr">
+        <is>
+          <t>full-time</t>
+        </is>
+      </c>
+      <c r="K871" s="719" t="inlineStr">
+        <is>
+          <t>$65k - $88k</t>
+        </is>
+      </c>
+      <c r="L871" s="720" t="n">
+        <v>46277</v>
+      </c>
+      <c r="M871" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N871" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O871" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P871" s="719" t="n"/>
+      <c r="Q871" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/desc/150747009818849333?ckey=Paid+Search+Manager&amp;rgn=55157&amp;pos=20&amp;groupId=41521&amp;elckey=-2609051204955160592&amp;p=1&amp;aq=-17202559000866049&amp;cid=19881&amp;jobAge=258&amp;brelb=15&amp;bscr=148.61942&amp;scr=148.61942</t>
+        </is>
+      </c>
+      <c r="R871" s="719" t="n"/>
+      <c r="S871" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T871" s="719" t="n"/>
+      <c r="U871" s="719" t="n"/>
+      <c r="V871" s="719" t="n"/>
+      <c r="W871" s="719" t="n"/>
+    </row>
+    <row r="872">
+      <c r="A872" s="719" t="n">
+        <v>871</v>
+      </c>
+      <c r="B872" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C872" s="719" t="inlineStr">
+        <is>
+          <t>Media Works</t>
+        </is>
+      </c>
+      <c r="D872" s="719" t="inlineStr">
+        <is>
+          <t>Paid Search Specialist</t>
+        </is>
+      </c>
+      <c r="E872" s="722" t="n">
+        <v>59</v>
+      </c>
+      <c r="F872" s="723" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G872" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H872" s="719" t="inlineStr">
+        <is>
+          <t>Baltimore, MD</t>
+        </is>
+      </c>
+      <c r="I872" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J872" s="719" t="n"/>
+      <c r="K872" s="719" t="n"/>
+      <c r="L872" s="720" t="n">
+        <v>46278</v>
+      </c>
+      <c r="M872" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N872" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O872" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P872" s="719" t="n"/>
+      <c r="Q872" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/desc/-3143928208055467601?ckey=Paid+Search+Specialist&amp;rgn=55157&amp;pos=8&amp;groupId=41016&amp;elckey=8367085328669080449&amp;p=1&amp;aq=-396050244561553006&amp;cid=19881&amp;jobAge=234&amp;brelb=110&amp;bscr=1596.6746&amp;scr=1596.6746</t>
+        </is>
+      </c>
+      <c r="R872" s="719" t="n"/>
+      <c r="S872" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T872" s="719" t="n"/>
+      <c r="U872" s="719" t="n"/>
+      <c r="V872" s="719" t="n"/>
+      <c r="W872" s="719" t="n"/>
+    </row>
+    <row r="873">
+      <c r="A873" s="719" t="n">
+        <v>872</v>
+      </c>
+      <c r="B873" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C873" s="719" t="inlineStr">
+        <is>
+          <t>Inizio Evoke</t>
+        </is>
+      </c>
+      <c r="D873" s="719" t="inlineStr">
+        <is>
+          <t>Paid Search Supervisor</t>
+        </is>
+      </c>
+      <c r="E873" s="722" t="n">
+        <v>44</v>
+      </c>
+      <c r="F873" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G873" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H873" s="719" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA</t>
+        </is>
+      </c>
+      <c r="I873" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J873" s="719" t="n"/>
+      <c r="K873" s="719" t="inlineStr">
+        <is>
+          <t>$100k - $120k</t>
+        </is>
+      </c>
+      <c r="L873" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M873" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N873" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O873" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P873" s="719" t="n"/>
+      <c r="Q873" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-3783512821330446431?p=1&amp;pos=9&amp;rgn=55157&amp;cid=19881&amp;ckey=Paid+Search+Specialist&amp;jobAge=39&amp;brelb=100&amp;scr=1446.7476&amp;bscr=1446.7476&amp;aq=-396050244561553006&amp;elckey=8367085328669080449</t>
+        </is>
+      </c>
+      <c r="R873" s="719" t="n"/>
+      <c r="S873" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T873" s="719" t="n"/>
+      <c r="U873" s="719" t="n"/>
+      <c r="V873" s="719" t="n"/>
+      <c r="W873" s="719" t="n"/>
+    </row>
+    <row r="874">
+      <c r="A874" s="719" t="n">
+        <v>873</v>
+      </c>
+      <c r="B874" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C874" s="719" t="inlineStr">
+        <is>
+          <t>CIGNA</t>
+        </is>
+      </c>
+      <c r="D874" s="719" t="inlineStr">
+        <is>
+          <t>Lead Analyst, Technical Search (SEO/AEO/GEO)</t>
+        </is>
+      </c>
+      <c r="E874" s="722" t="n">
+        <v>52</v>
+      </c>
+      <c r="F874" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G874" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H874" s="719" t="inlineStr">
+        <is>
+          <t>Bloomfield, CT</t>
+        </is>
+      </c>
+      <c r="I874" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J874" s="719" t="n"/>
+      <c r="K874" s="719" t="inlineStr">
+        <is>
+          <t>$79.1k - $131.8k</t>
+        </is>
+      </c>
+      <c r="L874" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M874" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N874" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O874" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P874" s="719" t="n"/>
+      <c r="Q874" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/7572799814767438644?p=1&amp;pos=18&amp;rgn=55157&amp;cid=19881&amp;ckey=Paid+Search+Specialist&amp;jobAge=63&amp;brelb=100&amp;scr=615.8714&amp;bscr=615.8714&amp;aq=-396050244561553006&amp;elckey=8367085328669080449</t>
+        </is>
+      </c>
+      <c r="R874" s="719" t="n"/>
+      <c r="S874" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T874" s="719" t="n"/>
+      <c r="U874" s="719" t="n"/>
+      <c r="V874" s="719" t="n"/>
+      <c r="W874" s="719" t="n"/>
+    </row>
+    <row r="875">
+      <c r="A875" s="719" t="n">
+        <v>874</v>
+      </c>
+      <c r="B875" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C875" s="719" t="inlineStr">
+        <is>
+          <t>Skybox Capital</t>
+        </is>
+      </c>
+      <c r="D875" s="719" t="inlineStr">
+        <is>
+          <t>Paid Search Analyst (Entry Level) - Go Tickets</t>
+        </is>
+      </c>
+      <c r="E875" s="722" t="n">
+        <v>49</v>
+      </c>
+      <c r="F875" s="723" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G875" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H875" s="719" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="I875" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J875" s="719" t="inlineStr">
+        <is>
+          <t>full-time</t>
+        </is>
+      </c>
+      <c r="K875" s="719" t="n"/>
+      <c r="L875" s="720" t="n">
+        <v>46224</v>
+      </c>
+      <c r="M875" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N875" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O875" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P875" s="719" t="n"/>
+      <c r="Q875" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/desc/-6343854235974185547?ckey=Paid+Search+Specialist&amp;rgn=55157&amp;pos=19&amp;groupId=41016&amp;elckey=8367085328669080449&amp;p=1&amp;aq=-396050244561553006&amp;cid=19881&amp;jobAge=1530&amp;brelb=100&amp;bscr=561.6406&amp;scr=561.6406</t>
+        </is>
+      </c>
+      <c r="R875" s="719" t="n"/>
+      <c r="S875" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T875" s="719" t="n"/>
+      <c r="U875" s="719" t="n"/>
+      <c r="V875" s="719" t="n"/>
+      <c r="W875" s="719" t="n"/>
+    </row>
+    <row r="876">
+      <c r="A876" s="719" t="n">
+        <v>875</v>
+      </c>
+      <c r="B876" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C876" s="719" t="inlineStr">
+        <is>
+          <t>Superior Executive Legal Recruiting</t>
+        </is>
+      </c>
+      <c r="D876" s="719" t="inlineStr">
+        <is>
+          <t>PPC Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E876" s="722" t="n">
+        <v>58</v>
+      </c>
+      <c r="F876" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G876" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H876" s="719" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I876" s="719" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="J876" s="719" t="n"/>
+      <c r="K876" s="719" t="n"/>
+      <c r="L876" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M876" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N876" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O876" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P876" s="719" t="n"/>
+      <c r="Q876" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/2814126476219348813?p=1&amp;pos=7&amp;rgn=55157&amp;cid=19881&amp;ckey=PPC+Manager&amp;jobAge=42&amp;brelb=10&amp;scr=207.71158&amp;bscr=207.71158&amp;aq=9023639601359958054&amp;elckey=-8560584423263407481</t>
+        </is>
+      </c>
+      <c r="R876" s="719" t="n"/>
+      <c r="S876" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T876" s="719" t="n"/>
+      <c r="U876" s="719" t="n"/>
+      <c r="V876" s="719" t="n"/>
+      <c r="W876" s="719" t="n"/>
+    </row>
+    <row r="877">
+      <c r="A877" s="719" t="n">
+        <v>876</v>
+      </c>
+      <c r="B877" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C877" s="719" t="inlineStr">
+        <is>
+          <t>Huzzle.com</t>
+        </is>
+      </c>
+      <c r="D877" s="719" t="inlineStr">
+        <is>
+          <t>Remote PPC Manager | High-ROI Paid Media Leader</t>
+        </is>
+      </c>
+      <c r="E877" s="722" t="n">
+        <v>64</v>
+      </c>
+      <c r="F877" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G877" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H877" s="719" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I877" s="719" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="J877" s="719" t="n"/>
+      <c r="K877" s="719" t="n"/>
+      <c r="L877" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M877" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N877" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O877" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P877" s="719" t="n"/>
+      <c r="Q877" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/2218180771029220984?p=1&amp;pos=9&amp;rgn=55157&amp;cid=19881&amp;ckey=PPC+Manager&amp;jobAge=90&amp;brelb=10&amp;scr=183.83502&amp;bscr=183.83502&amp;aq=9023639601359958054&amp;elckey=-8560584423263407481</t>
+        </is>
+      </c>
+      <c r="R877" s="719" t="n"/>
+      <c r="S877" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T877" s="719" t="n"/>
+      <c r="U877" s="719" t="n"/>
+      <c r="V877" s="719" t="n"/>
+      <c r="W877" s="719" t="n"/>
+    </row>
+    <row r="878">
+      <c r="A878" s="719" t="n">
+        <v>877</v>
+      </c>
+      <c r="B878" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C878" s="719" t="inlineStr">
+        <is>
+          <t>Audacy</t>
+        </is>
+      </c>
+      <c r="D878" s="719" t="inlineStr">
+        <is>
+          <t>Search Engine Marketing (SEM) Account Manager</t>
+        </is>
+      </c>
+      <c r="E878" s="722" t="n">
+        <v>45</v>
+      </c>
+      <c r="F878" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G878" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H878" s="719" t="inlineStr">
+        <is>
+          <t>Chattanooga, TN</t>
+        </is>
+      </c>
+      <c r="I878" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J878" s="719" t="n"/>
+      <c r="K878" s="719" t="inlineStr">
+        <is>
+          <t>$55k - $65k</t>
+        </is>
+      </c>
+      <c r="L878" s="720" t="n">
+        <v>46283</v>
+      </c>
+      <c r="M878" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N878" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O878" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P878" s="719" t="n"/>
+      <c r="Q878" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/5054035278756328357?p=1&amp;pos=2&amp;rgn=55157&amp;cid=19881&amp;ckey=SEM+Manager&amp;jobAge=107&amp;brelb=100&amp;scr=728.2281&amp;bscr=728.2281&amp;aq=8355652149010879591&amp;elckey=-8283006412667774407</t>
+        </is>
+      </c>
+      <c r="R878" s="719" t="n"/>
+      <c r="S878" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T878" s="719" t="n"/>
+      <c r="U878" s="719" t="n"/>
+      <c r="V878" s="719" t="n"/>
+      <c r="W878" s="719" t="n"/>
+    </row>
+    <row r="879">
+      <c r="A879" s="719" t="n">
+        <v>878</v>
+      </c>
+      <c r="B879" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C879" s="719" t="inlineStr">
+        <is>
+          <t>Capital Square LLC</t>
+        </is>
+      </c>
+      <c r="D879" s="719" t="inlineStr">
+        <is>
+          <t>Regional Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E879" s="722" t="n">
+        <v>57</v>
+      </c>
+      <c r="F879" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G879" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H879" s="719" t="inlineStr">
+        <is>
+          <t>Glen Allen, VA</t>
+        </is>
+      </c>
+      <c r="I879" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J879" s="719" t="n"/>
+      <c r="K879" s="719" t="inlineStr">
+        <is>
+          <t>$75k - $85k</t>
+        </is>
+      </c>
+      <c r="L879" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M879" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N879" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O879" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P879" s="719" t="n"/>
+      <c r="Q879" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/559778930561099862?p=1&amp;pos=11&amp;rgn=55157&amp;cid=19881&amp;ckey=SEM+Manager&amp;jobAge=90&amp;brelb=10&amp;scr=223.7824&amp;bscr=223.7824&amp;aq=8355652149010879591&amp;elckey=-8283006412667774407</t>
+        </is>
+      </c>
+      <c r="R879" s="719" t="n"/>
+      <c r="S879" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T879" s="719" t="n"/>
+      <c r="U879" s="719" t="n"/>
+      <c r="V879" s="719" t="n"/>
+      <c r="W879" s="719" t="n"/>
+    </row>
+    <row r="880">
+      <c r="A880" s="719" t="n">
+        <v>879</v>
+      </c>
+      <c r="B880" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C880" s="719" t="inlineStr">
+        <is>
+          <t>Doordash</t>
+        </is>
+      </c>
+      <c r="D880" s="719" t="inlineStr">
+        <is>
+          <t>Associate Manager, Consumer Integrated Marketing - New Verticals Habituation</t>
+        </is>
+      </c>
+      <c r="E880" s="722" t="n">
+        <v>56</v>
+      </c>
+      <c r="F880" s="723" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G880" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H880" s="719" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="I880" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J880" s="719" t="n"/>
+      <c r="K880" s="719" t="inlineStr">
+        <is>
+          <t>$108.8k - $160k</t>
+        </is>
+      </c>
+      <c r="L880" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M880" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N880" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O880" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P880" s="719" t="n"/>
+      <c r="Q880" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-8687328179435497866?p=1&amp;pos=17&amp;rgn=55157&amp;cid=19881&amp;ckey=SEM+Manager&amp;jobAge=66&amp;brelb=100&amp;scr=186.7872&amp;bscr=186.7872&amp;aq=8355652149010879591&amp;elckey=-8283006412667774407</t>
+        </is>
+      </c>
+      <c r="R880" s="719" t="n"/>
+      <c r="S880" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T880" s="719" t="n"/>
+      <c r="U880" s="719" t="n"/>
+      <c r="V880" s="719" t="n"/>
+      <c r="W880" s="719" t="n"/>
+    </row>
+    <row r="881">
+      <c r="A881" s="719" t="n">
+        <v>880</v>
+      </c>
+      <c r="B881" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C881" s="719" t="inlineStr">
+        <is>
+          <t>Chartis Interactive</t>
+        </is>
+      </c>
+      <c r="D881" s="719" t="inlineStr">
+        <is>
+          <t>Digital Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E881" s="722" t="n">
+        <v>56</v>
+      </c>
+      <c r="F881" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G881" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H881" s="719" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I881" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J881" s="719" t="n"/>
+      <c r="K881" s="719" t="n"/>
+      <c r="L881" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M881" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N881" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O881" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P881" s="719" t="n"/>
+      <c r="Q881" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/6798747860686555146?p=1&amp;pos=19&amp;rgn=55157&amp;cid=19881&amp;ckey=Digital+Marketing+Manager&amp;jobAge=42&amp;brelb=10&amp;scr=186.99078&amp;bscr=186.99078&amp;aq=-1311798429678385746&amp;elckey=-6422506978848355027</t>
+        </is>
+      </c>
+      <c r="R881" s="719" t="n"/>
+      <c r="S881" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T881" s="719" t="n"/>
+      <c r="U881" s="719" t="n"/>
+      <c r="V881" s="719" t="n"/>
+      <c r="W881" s="719" t="n"/>
+    </row>
+    <row r="882">
+      <c r="A882" s="719" t="n">
+        <v>881</v>
+      </c>
+      <c r="B882" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C882" s="719" t="inlineStr">
+        <is>
+          <t>Socket</t>
+        </is>
+      </c>
+      <c r="D882" s="719" t="inlineStr">
+        <is>
+          <t>Senior Paid Media Manager</t>
+        </is>
+      </c>
+      <c r="E882" s="722" t="n">
+        <v>52</v>
+      </c>
+      <c r="F882" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G882" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H882" s="719" t="inlineStr">
+        <is>
+          <t>Murray, UT</t>
+        </is>
+      </c>
+      <c r="I882" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J882" s="719" t="n"/>
+      <c r="K882" s="719" t="n"/>
+      <c r="L882" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="M882" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N882" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O882" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P882" s="719" t="n"/>
+      <c r="Q882" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-4639457595483415693?p=1&amp;pos=1&amp;rgn=45&amp;cid=19881&amp;ckey=Paid+Media+Manager&amp;brelb=10&amp;scr=848.58795&amp;bscr=848.58795&amp;aq=4600203927708708134&amp;elckey=-3776736543079247748</t>
+        </is>
+      </c>
+      <c r="R882" s="719" t="n"/>
+      <c r="S882" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T882" s="719" t="n"/>
+      <c r="U882" s="719" t="n"/>
+      <c r="V882" s="719" t="n"/>
+      <c r="W882" s="719" t="n"/>
+    </row>
+    <row r="883">
+      <c r="A883" s="719" t="n">
+        <v>882</v>
+      </c>
+      <c r="B883" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C883" s="719" t="inlineStr">
+        <is>
+          <t>Torus</t>
+        </is>
+      </c>
+      <c r="D883" s="719" t="inlineStr">
+        <is>
+          <t>Product Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E883" s="722" t="n">
+        <v>43</v>
+      </c>
+      <c r="F883" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G883" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H883" s="719" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="I883" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J883" s="719" t="n"/>
+      <c r="K883" s="719" t="inlineStr">
+        <is>
+          <t>$165k - $190k</t>
+        </is>
+      </c>
+      <c r="L883" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M883" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N883" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O883" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P883" s="719" t="n"/>
+      <c r="Q883" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/813402454918400979?p=1&amp;pos=19&amp;rgn=45&amp;cid=19881&amp;ckey=Paid+Media+Manager&amp;jobAge=19&amp;brelb=10&amp;scr=104.5355&amp;bscr=104.5355&amp;aq=4600203927708708134&amp;elckey=-3776736543079247748</t>
+        </is>
+      </c>
+      <c r="R883" s="719" t="n"/>
+      <c r="S883" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T883" s="719" t="n"/>
+      <c r="U883" s="719" t="n"/>
+      <c r="V883" s="719" t="n"/>
+      <c r="W883" s="719" t="n"/>
+    </row>
+    <row r="884">
+      <c r="A884" s="719" t="n">
+        <v>883</v>
+      </c>
+      <c r="B884" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C884" s="719" t="inlineStr">
+        <is>
+          <t>Sunco Lighting</t>
+        </is>
+      </c>
+      <c r="D884" s="719" t="inlineStr">
+        <is>
+          <t>Senior Paid Media Manager</t>
+        </is>
+      </c>
+      <c r="E884" s="722" t="n">
+        <v>41</v>
+      </c>
+      <c r="F884" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G884" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H884" s="719" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="I884" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J884" s="719" t="n"/>
+      <c r="K884" s="719" t="n"/>
+      <c r="L884" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M884" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N884" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O884" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P884" s="719" t="n"/>
+      <c r="Q884" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/2134474442812066608?p=1&amp;pos=13&amp;rgn=55157&amp;cid=19881&amp;ckey=Paid+Media+Manager&amp;jobAge=90&amp;brelb=10&amp;scr=832.5565&amp;bscr=832.5565&amp;aq=7337777505112425399&amp;elckey=2653251887168839570</t>
+        </is>
+      </c>
+      <c r="R884" s="719" t="n"/>
+      <c r="S884" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T884" s="719" t="n"/>
+      <c r="U884" s="719" t="n"/>
+      <c r="V884" s="719" t="n"/>
+      <c r="W884" s="719" t="n"/>
+    </row>
+    <row r="885">
+      <c r="A885" s="719" t="n">
+        <v>884</v>
+      </c>
+      <c r="B885" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C885" s="719" t="inlineStr">
+        <is>
+          <t>Loadsmart</t>
+        </is>
+      </c>
+      <c r="D885" s="719" t="inlineStr">
+        <is>
+          <t>Senior Paid Media Manager (Enterprise B2B)</t>
+        </is>
+      </c>
+      <c r="E885" s="722" t="n">
+        <v>23</v>
+      </c>
+      <c r="F885" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G885" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H885" s="719" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="I885" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J885" s="719" t="n"/>
+      <c r="K885" s="719" t="inlineStr">
+        <is>
+          <t>$120k - $140k</t>
+        </is>
+      </c>
+      <c r="L885" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M885" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N885" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O885" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P885" s="719" t="n"/>
+      <c r="Q885" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/2839178670932466016?p=1&amp;pos=20&amp;rgn=55157&amp;cid=19881&amp;ckey=Paid+Media+Manager&amp;jobAge=39&amp;brelb=100&amp;scr=821.99365&amp;bscr=821.99365&amp;aq=7337777505112425399&amp;elckey=2653251887168839570</t>
+        </is>
+      </c>
+      <c r="R885" s="719" t="n"/>
+      <c r="S885" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T885" s="719" t="n"/>
+      <c r="U885" s="719" t="n"/>
+      <c r="V885" s="719" t="n"/>
+      <c r="W885" s="719" t="n"/>
+    </row>
+    <row r="886">
+      <c r="A886" s="719" t="n">
+        <v>885</v>
+      </c>
+      <c r="B886" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C886" s="719" t="inlineStr">
+        <is>
+          <t>Private Wealth Law Group</t>
+        </is>
+      </c>
+      <c r="D886" s="719" t="inlineStr">
+        <is>
+          <t>Senior Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E886" s="722" t="n">
+        <v>50</v>
+      </c>
+      <c r="F886" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G886" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H886" s="719" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="I886" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J886" s="719" t="n"/>
+      <c r="K886" s="719" t="n"/>
+      <c r="L886" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="M886" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N886" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O886" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P886" s="719" t="n"/>
+      <c r="Q886" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/1504600378239043648?p=1&amp;pos=4&amp;rgn=45&amp;cid=19881&amp;ckey=Search+Marketing+Manager&amp;jobAge=1&amp;brelb=10&amp;scr=237.98851&amp;bscr=237.98851&amp;aq=4672009537455359971&amp;elckey=5500712979101207184</t>
+        </is>
+      </c>
+      <c r="R886" s="719" t="n"/>
+      <c r="S886" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T886" s="719" t="n"/>
+      <c r="U886" s="719" t="n"/>
+      <c r="V886" s="719" t="n"/>
+      <c r="W886" s="719" t="n"/>
+    </row>
+    <row r="887">
+      <c r="A887" s="719" t="n">
+        <v>886</v>
+      </c>
+      <c r="B887" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C887" s="719" t="inlineStr">
+        <is>
+          <t>Backcountry.com</t>
+        </is>
+      </c>
+      <c r="D887" s="719" t="inlineStr">
+        <is>
+          <t>Vice President, Performance Marketing</t>
+        </is>
+      </c>
+      <c r="E887" s="722" t="n">
+        <v>58</v>
+      </c>
+      <c r="F887" s="723" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G887" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H887" s="719" t="inlineStr">
+        <is>
+          <t>Cottonwood Heights, UT</t>
+        </is>
+      </c>
+      <c r="I887" s="719" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="J887" s="719" t="n"/>
+      <c r="K887" s="719" t="n"/>
+      <c r="L887" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="M887" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N887" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O887" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P887" s="719" t="n"/>
+      <c r="Q887" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-6834277330776592927?p=1&amp;pos=16&amp;rgn=45&amp;cid=19881&amp;ckey=Search+Marketing+Manager&amp;jobAge=1&amp;brelb=10&amp;scr=152.94914&amp;bscr=152.94914&amp;aq=4672009537455359971&amp;elckey=5500712979101207184</t>
+        </is>
+      </c>
+      <c r="R887" s="719" t="n"/>
+      <c r="S887" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T887" s="719" t="n"/>
+      <c r="U887" s="719" t="n"/>
+      <c r="V887" s="719" t="n"/>
+      <c r="W887" s="719" t="n"/>
+    </row>
+    <row r="888">
+      <c r="A888" s="719" t="n">
+        <v>887</v>
+      </c>
+      <c r="B888" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C888" s="719" t="inlineStr">
+        <is>
+          <t>Colling Media</t>
+        </is>
+      </c>
+      <c r="D888" s="719" t="inlineStr">
+        <is>
+          <t>Search Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E888" s="722" t="n">
+        <v>50</v>
+      </c>
+      <c r="F888" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G888" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H888" s="719" t="inlineStr">
+        <is>
+          <t>Phoenix, AZ</t>
+        </is>
+      </c>
+      <c r="I888" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J888" s="719" t="n"/>
+      <c r="K888" s="719" t="n"/>
+      <c r="L888" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="M888" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N888" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O888" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P888" s="719" t="n"/>
+      <c r="Q888" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/7972828035650362887?p=1&amp;pos=20&amp;rgn=55157&amp;cid=19881&amp;ckey=Search+Marketing+Manager&amp;jobAge=18&amp;brelb=10&amp;scr=888.94604&amp;bscr=888.94604&amp;aq=-4387840855259045464&amp;elckey=-5129356719772902906</t>
+        </is>
+      </c>
+      <c r="R888" s="719" t="n"/>
+      <c r="S888" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T888" s="719" t="n"/>
+      <c r="U888" s="719" t="n"/>
+      <c r="V888" s="719" t="n"/>
+      <c r="W888" s="719" t="n"/>
+    </row>
+    <row r="889">
+      <c r="A889" s="719" t="n">
+        <v>888</v>
+      </c>
+      <c r="B889" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C889" s="719" t="inlineStr">
+        <is>
+          <t>CHG Healthcare</t>
+        </is>
+      </c>
+      <c r="D889" s="719" t="inlineStr">
+        <is>
+          <t>Growth Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E889" s="722" t="n">
+        <v>65</v>
+      </c>
+      <c r="F889" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G889" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H889" s="719" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="I889" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J889" s="719" t="n"/>
+      <c r="K889" s="719" t="inlineStr">
+        <is>
+          <t>$92.9k - $179.7k</t>
+        </is>
+      </c>
+      <c r="L889" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M889" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N889" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O889" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P889" s="719" t="n"/>
+      <c r="Q889" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-7700046342209133715?p=1&amp;pos=3&amp;rgn=45&amp;cid=19881&amp;ckey=Marketing+Analytics+Manager&amp;jobAge=90&amp;brelb=10&amp;scr=302.25763&amp;bscr=302.25763&amp;aq=-3650539951949601963&amp;elckey=862103136135905967</t>
+        </is>
+      </c>
+      <c r="R889" s="719" t="n"/>
+      <c r="S889" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T889" s="719" t="n"/>
+      <c r="U889" s="719" t="n"/>
+      <c r="V889" s="719" t="inlineStr">
+        <is>
+          <t>file:///C:/Users/DCALL/Desktop/gecko/output/resumes/Dave-Call%2BCHG-Healthcare%2B5846006026.docx</t>
+        </is>
+      </c>
+      <c r="W889" s="719" t="n"/>
+    </row>
+    <row r="890">
+      <c r="A890" s="719" t="n">
+        <v>889</v>
+      </c>
+      <c r="B890" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C890" s="719" t="inlineStr">
+        <is>
+          <t>CallTower</t>
+        </is>
+      </c>
+      <c r="D890" s="719" t="inlineStr">
+        <is>
+          <t>Marketing Operations Manager</t>
+        </is>
+      </c>
+      <c r="E890" s="722" t="n">
+        <v>26</v>
+      </c>
+      <c r="F890" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G890" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H890" s="719" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="I890" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J890" s="719" t="n"/>
+      <c r="K890" s="719" t="n"/>
+      <c r="L890" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M890" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N890" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O890" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P890" s="719" t="n"/>
+      <c r="Q890" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-7956507514248360616?p=1&amp;pos=17&amp;rgn=45&amp;cid=19881&amp;ckey=Marketing+Analytics+Manager&amp;jobAge=66&amp;brelb=10&amp;scr=213.84218&amp;bscr=213.84218&amp;aq=-3650539951949601963&amp;elckey=862103136135905967</t>
+        </is>
+      </c>
+      <c r="R890" s="719" t="n"/>
+      <c r="S890" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T890" s="719" t="n"/>
+      <c r="U890" s="719" t="n"/>
+      <c r="V890" s="719" t="n"/>
+      <c r="W890" s="719" t="n"/>
+    </row>
+    <row r="891">
+      <c r="A891" s="719" t="n">
+        <v>890</v>
+      </c>
+      <c r="B891" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C891" s="719" t="inlineStr">
+        <is>
+          <t>NeoGenomics</t>
+        </is>
+      </c>
+      <c r="D891" s="719" t="inlineStr">
+        <is>
+          <t>Marketing Analytics Manager</t>
+        </is>
+      </c>
+      <c r="E891" s="722" t="n">
+        <v>62</v>
+      </c>
+      <c r="F891" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G891" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H891" s="719" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I891" s="719" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="J891" s="719" t="n"/>
+      <c r="K891" s="719" t="n"/>
+      <c r="L891" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="M891" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N891" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O891" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P891" s="719" t="n"/>
+      <c r="Q891" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/7207818852323698094?p=1&amp;pos=8&amp;rgn=55157&amp;cid=19881&amp;ckey=Marketing+Analytics+Manager&amp;jobAge=1&amp;brelb=10&amp;scr=2470.037&amp;bscr=2470.037&amp;aq=5043476973562925237&amp;elckey=4338690561863893485</t>
+        </is>
+      </c>
+      <c r="R891" s="719" t="n"/>
+      <c r="S891" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T891" s="719" t="n"/>
+      <c r="U891" s="719" t="n"/>
+      <c r="V891" s="719" t="n"/>
+      <c r="W891" s="719" t="n"/>
+    </row>
+    <row r="892">
+      <c r="A892" s="719" t="n">
+        <v>891</v>
+      </c>
+      <c r="B892" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C892" s="719" t="inlineStr">
+        <is>
+          <t>GrabJobs</t>
+        </is>
+      </c>
+      <c r="D892" s="719" t="inlineStr">
+        <is>
+          <t>Marketing Analytics Manager</t>
+        </is>
+      </c>
+      <c r="E892" s="722" t="n">
+        <v>59</v>
+      </c>
+      <c r="F892" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G892" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H892" s="719" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale, FL</t>
+        </is>
+      </c>
+      <c r="I892" s="719" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="J892" s="719" t="n"/>
+      <c r="K892" s="719" t="n"/>
+      <c r="L892" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M892" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N892" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O892" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P892" s="719" t="n"/>
+      <c r="Q892" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-3862913434670880683?p=1&amp;pos=11&amp;rgn=55157&amp;cid=19881&amp;ckey=Marketing+Analytics+Manager&amp;jobAge=42&amp;brelb=10&amp;scr=2450.7495&amp;bscr=2450.7495&amp;aq=5043476973562925237&amp;elckey=4338690561863893485</t>
+        </is>
+      </c>
+      <c r="R892" s="719" t="n"/>
+      <c r="S892" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T892" s="719" t="n"/>
+      <c r="U892" s="719" t="n"/>
+      <c r="V892" s="719" t="n"/>
+      <c r="W892" s="719" t="n"/>
+    </row>
+    <row r="893">
+      <c r="A893" s="719" t="n">
+        <v>892</v>
+      </c>
+      <c r="B893" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C893" s="719" t="inlineStr">
+        <is>
+          <t>Twilio</t>
+        </is>
+      </c>
+      <c r="D893" s="719" t="inlineStr">
+        <is>
+          <t>Sr. Marketing Strategy and Analytics Manager</t>
+        </is>
+      </c>
+      <c r="E893" s="722" t="n">
+        <v>35</v>
+      </c>
+      <c r="F893" s="723" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G893" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H893" s="719" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="I893" s="719" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="J893" s="719" t="inlineStr">
+        <is>
+          <t>full-time</t>
+        </is>
+      </c>
+      <c r="K893" s="719" t="n"/>
+      <c r="L893" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M893" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N893" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O893" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P893" s="719" t="n"/>
+      <c r="Q893" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/desc/3912355311191622548?ckey=Marketing+Analytics+Manager&amp;rgn=55157&amp;pos=16&amp;groupId=-1925849718&amp;elckey=4338690561863893485&amp;p=1&amp;aq=5043476973562925237&amp;cid=19881&amp;jobAge=90&amp;brelb=15&amp;bscr=1589.7133&amp;scr=1589.7133</t>
+        </is>
+      </c>
+      <c r="R893" s="719" t="n"/>
+      <c r="S893" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T893" s="719" t="n"/>
+      <c r="U893" s="719" t="n"/>
+      <c r="V893" s="719" t="n"/>
+      <c r="W893" s="719" t="n"/>
+    </row>
+    <row r="894">
+      <c r="A894" s="719" t="n">
+        <v>893</v>
+      </c>
+      <c r="B894" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C894" s="719" t="inlineStr">
+        <is>
+          <t>&amp;Barr</t>
+        </is>
+      </c>
+      <c r="D894" s="719" t="inlineStr">
+        <is>
+          <t>Director of Digital Marketing &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="E894" s="722" t="n">
+        <v>52</v>
+      </c>
+      <c r="F894" s="723" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G894" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H894" s="719" t="inlineStr">
+        <is>
+          <t>Orlando, FL</t>
+        </is>
+      </c>
+      <c r="I894" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J894" s="719" t="n"/>
+      <c r="K894" s="719" t="n"/>
+      <c r="L894" s="720" t="n">
+        <v>46281</v>
+      </c>
+      <c r="M894" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N894" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O894" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P894" s="719" t="n"/>
+      <c r="Q894" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/desc/6505045710150425240?ckey=Marketing+Analytics+Manager&amp;rgn=55157&amp;pos=18&amp;groupId=-1925849718&amp;elckey=4338690561863893485&amp;p=1&amp;aq=5043476973562925237&amp;cid=19881&amp;jobAge=162&amp;brelb=15&amp;bscr=875.28125&amp;scr=875.28125</t>
+        </is>
+      </c>
+      <c r="R894" s="719" t="n"/>
+      <c r="S894" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T894" s="719" t="n"/>
+      <c r="U894" s="719" t="n"/>
+      <c r="V894" s="719" t="n"/>
+      <c r="W894" s="719" t="n"/>
+    </row>
+    <row r="895">
+      <c r="A895" s="719" t="n">
+        <v>894</v>
+      </c>
+      <c r="B895" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C895" s="719" t="inlineStr">
+        <is>
+          <t>Forsyth Barnes</t>
+        </is>
+      </c>
+      <c r="D895" s="719" t="inlineStr">
+        <is>
+          <t>Digital Marketing Analyst</t>
+        </is>
+      </c>
+      <c r="E895" s="722" t="n">
+        <v>48</v>
+      </c>
+      <c r="F895" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G895" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H895" s="719" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="I895" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J895" s="719" t="n"/>
+      <c r="K895" s="719" t="n"/>
+      <c r="L895" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="M895" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N895" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O895" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P895" s="719" t="n"/>
+      <c r="Q895" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-705539290782970174?p=1&amp;pos=8&amp;rgn=55157&amp;cid=19881&amp;ckey=Digital+Marketing+Analyst&amp;jobAge=1&amp;brelb=10&amp;scr=2253.8088&amp;bscr=2253.8088&amp;aq=8034963705413381549&amp;elckey=5783322791353163661</t>
+        </is>
+      </c>
+      <c r="R895" s="719" t="n"/>
+      <c r="S895" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T895" s="719" t="n"/>
+      <c r="U895" s="719" t="n"/>
+      <c r="V895" s="719" t="n"/>
+      <c r="W895" s="719" t="n"/>
+    </row>
+    <row r="896">
+      <c r="A896" s="719" t="n">
+        <v>895</v>
+      </c>
+      <c r="B896" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C896" s="719" t="inlineStr">
+        <is>
+          <t>CMI Media and Compas</t>
+        </is>
+      </c>
+      <c r="D896" s="719" t="inlineStr">
+        <is>
+          <t>Analyst, Digital Marketing Analytics</t>
+        </is>
+      </c>
+      <c r="E896" s="722" t="n">
+        <v>52</v>
+      </c>
+      <c r="F896" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G896" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H896" s="719" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="I896" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J896" s="719" t="n"/>
+      <c r="K896" s="719" t="inlineStr">
+        <is>
+          <t>$40k - $75k</t>
+        </is>
+      </c>
+      <c r="L896" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M896" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N896" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O896" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P896" s="719" t="n"/>
+      <c r="Q896" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-1274261719067460536?p=1&amp;pos=20&amp;rgn=55157&amp;cid=19881&amp;ckey=Digital+Marketing+Analyst&amp;jobAge=90&amp;brelb=100&amp;scr=376.89413&amp;bscr=376.89413&amp;aq=8034963705413381549&amp;elckey=5783322791353163661</t>
+        </is>
+      </c>
+      <c r="R896" s="719" t="n"/>
+      <c r="S896" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T896" s="719" t="n"/>
+      <c r="U896" s="719" t="n"/>
+      <c r="V896" s="719" t="n"/>
+      <c r="W896" s="719" t="n"/>
+    </row>
+    <row r="897">
+      <c r="A897" s="719" t="n">
+        <v>896</v>
+      </c>
+      <c r="B897" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C897" s="719" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D897" s="719" t="inlineStr">
+        <is>
+          <t>Growth Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E897" s="722" t="n">
+        <v>67</v>
+      </c>
+      <c r="F897" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G897" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H897" s="719" t="inlineStr">
+        <is>
+          <t>Lehi, UT</t>
+        </is>
+      </c>
+      <c r="I897" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J897" s="719" t="n"/>
+      <c r="K897" s="719" t="n"/>
+      <c r="L897" s="720" t="n">
+        <v>46276</v>
+      </c>
+      <c r="M897" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N897" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O897" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P897" s="719" t="n"/>
+      <c r="Q897" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/desc/4277285931540338385?ckey=Growth+Marketing+Manager&amp;rgn=45&amp;pos=9&amp;groupId=1810086807&amp;elckey=-3949613940002492999&amp;p=1&amp;aq=-4345824593601355655&amp;cid=19881&amp;jobAge=282&amp;brelb=110&amp;bscr=236.69257&amp;scr=236.69257</t>
+        </is>
+      </c>
+      <c r="R897" s="719" t="n"/>
+      <c r="S897" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T897" s="719" t="n"/>
+      <c r="U897" s="719" t="n"/>
+      <c r="V897" s="719" t="n"/>
+      <c r="W897" s="719" t="n"/>
+    </row>
+    <row r="898">
+      <c r="A898" s="719" t="n">
+        <v>897</v>
+      </c>
+      <c r="B898" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C898" s="719" t="inlineStr">
+        <is>
+          <t>GrabJobs</t>
+        </is>
+      </c>
+      <c r="D898" s="719" t="inlineStr">
+        <is>
+          <t>Remote Channel Marketing Manager</t>
+        </is>
+      </c>
+      <c r="E898" s="722" t="n">
+        <v>40</v>
+      </c>
+      <c r="F898" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G898" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H898" s="719" t="inlineStr">
+        <is>
+          <t>Orem, UT</t>
+        </is>
+      </c>
+      <c r="I898" s="719" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="J898" s="719" t="n"/>
+      <c r="K898" s="719" t="n"/>
+      <c r="L898" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M898" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N898" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O898" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P898" s="719" t="n"/>
+      <c r="Q898" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/4034709652039652813?p=1&amp;pos=7&amp;rgn=45&amp;cid=19881&amp;ckey=E-Commerce+Marketing+Manager&amp;jobAge=66&amp;brelb=10&amp;scr=250.51628&amp;bscr=250.51628&amp;aq=7189496538214754252&amp;elckey=-5972005269433951653</t>
+        </is>
+      </c>
+      <c r="R898" s="719" t="n"/>
+      <c r="S898" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T898" s="719" t="n"/>
+      <c r="U898" s="719" t="n"/>
+      <c r="V898" s="719" t="n"/>
+      <c r="W898" s="719" t="n"/>
+    </row>
+    <row r="899">
+      <c r="A899" s="719" t="n">
+        <v>898</v>
+      </c>
+      <c r="B899" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C899" s="719" t="inlineStr">
+        <is>
+          <t>gleanwork</t>
+        </is>
+      </c>
+      <c r="D899" s="719" t="inlineStr">
+        <is>
+          <t>Senior Demand Generation Manager</t>
+        </is>
+      </c>
+      <c r="E899" s="722" t="n">
+        <v>58</v>
+      </c>
+      <c r="F899" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G899" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H899" s="719" t="inlineStr">
+        <is>
+          <t>Mountain View, CA</t>
+        </is>
+      </c>
+      <c r="I899" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J899" s="719" t="n"/>
+      <c r="K899" s="719" t="inlineStr">
+        <is>
+          <t>$163k - $187k</t>
+        </is>
+      </c>
+      <c r="L899" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M899" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N899" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O899" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P899" s="719" t="n"/>
+      <c r="Q899" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/1136621718323498624?p=1&amp;pos=19&amp;rgn=55157&amp;cid=19881&amp;ckey=Demand+Generation+Manager&amp;jobAge=91&amp;brelb=10&amp;scr=166.13522&amp;bscr=166.13522&amp;aq=4063026109195332817&amp;elckey=1817209552898100899</t>
+        </is>
+      </c>
+      <c r="R899" s="719" t="n"/>
+      <c r="S899" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T899" s="719" t="n"/>
+      <c r="U899" s="719" t="n"/>
+      <c r="V899" s="719" t="n"/>
+      <c r="W899" s="719" t="n"/>
+    </row>
+    <row r="900">
+      <c r="A900" s="719" t="n">
+        <v>899</v>
+      </c>
+      <c r="B900" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C900" s="719" t="inlineStr">
+        <is>
+          <t>Employ Inc.</t>
+        </is>
+      </c>
+      <c r="D900" s="719" t="inlineStr">
+        <is>
+          <t>Demand Generation Manager</t>
+        </is>
+      </c>
+      <c r="E900" s="722" t="n">
+        <v>58</v>
+      </c>
+      <c r="F900" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G900" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H900" s="719" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I900" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J900" s="719" t="n"/>
+      <c r="K900" s="719" t="inlineStr">
+        <is>
+          <t>$75.02k - $90k</t>
+        </is>
+      </c>
+      <c r="L900" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M900" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N900" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O900" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P900" s="719" t="n"/>
+      <c r="Q900" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-692844490951771382?p=1&amp;pos=20&amp;rgn=55157&amp;cid=19881&amp;ckey=Demand+Generation+Manager&amp;jobAge=19&amp;brelb=10&amp;scr=166.13522&amp;bscr=166.13522&amp;aq=4063026109195332817&amp;elckey=1817209552898100899</t>
+        </is>
+      </c>
+      <c r="R900" s="719" t="n"/>
+      <c r="S900" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T900" s="719" t="n"/>
+      <c r="U900" s="719" t="n"/>
+      <c r="V900" s="719" t="n"/>
+      <c r="W900" s="719" t="n"/>
+    </row>
+    <row r="901">
+      <c r="A901" s="719" t="n">
+        <v>900</v>
+      </c>
+      <c r="B901" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C901" s="719" t="inlineStr">
+        <is>
+          <t>SIA</t>
+        </is>
+      </c>
+      <c r="D901" s="719" t="inlineStr">
+        <is>
+          <t>Sr. Paid Search &amp; Paid Social Strategist</t>
+        </is>
+      </c>
+      <c r="E901" s="722" t="n">
+        <v>55</v>
+      </c>
+      <c r="F901" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G901" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H901" s="719" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="I901" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J901" s="719" t="n"/>
+      <c r="K901" s="719" t="inlineStr">
+        <is>
+          <t>$110k - $120k</t>
+        </is>
+      </c>
+      <c r="L901" s="720" t="n">
+        <v>46284</v>
+      </c>
+      <c r="M901" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N901" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O901" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P901" s="719" t="n"/>
+      <c r="Q901" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/3919374004369881660?p=1&amp;pos=4&amp;rgn=55157&amp;cid=19881&amp;ckey=Senior+Paid+Search+Strategist&amp;jobAge=91&amp;brelb=10&amp;scr=14378.07&amp;bscr=14378.07&amp;aq=-427099300053651923&amp;elckey=5303113098520002782</t>
+        </is>
+      </c>
+      <c r="R901" s="719" t="n"/>
+      <c r="S901" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T901" s="719" t="n"/>
+      <c r="U901" s="719" t="n"/>
+      <c r="V901" s="719" t="n"/>
+      <c r="W901" s="719" t="n"/>
+    </row>
+    <row r="902">
+      <c r="A902" s="719" t="n">
+        <v>901</v>
+      </c>
+      <c r="B902" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C902" s="719" t="inlineStr">
+        <is>
+          <t>Hurrdat</t>
+        </is>
+      </c>
+      <c r="D902" s="719" t="inlineStr">
+        <is>
+          <t>Paid Search Strategist</t>
+        </is>
+      </c>
+      <c r="E902" s="722" t="n">
+        <v>59</v>
+      </c>
+      <c r="F902" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G902" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H902" s="719" t="inlineStr">
+        <is>
+          <t>Lincoln, NE</t>
+        </is>
+      </c>
+      <c r="I902" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J902" s="719" t="n"/>
+      <c r="K902" s="719" t="n"/>
+      <c r="L902" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M902" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N902" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O902" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P902" s="719" t="n"/>
+      <c r="Q902" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-6874075858538672026?p=1&amp;pos=12&amp;rgn=55157&amp;cid=19881&amp;ckey=Senior+Paid+Search+Strategist&amp;jobAge=67&amp;brelb=100&amp;scr=4932.9536&amp;bscr=4932.9536&amp;aq=-427099300053651923&amp;elckey=5303113098520002782</t>
+        </is>
+      </c>
+      <c r="R902" s="719" t="n"/>
+      <c r="S902" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T902" s="719" t="n"/>
+      <c r="U902" s="719" t="n"/>
+      <c r="V902" s="719" t="n"/>
+      <c r="W902" s="719" t="n"/>
+    </row>
+    <row r="903">
+      <c r="A903" s="719" t="n">
+        <v>902</v>
+      </c>
+      <c r="B903" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C903" s="719" t="inlineStr">
+        <is>
+          <t>ONDA USA</t>
+        </is>
+      </c>
+      <c r="D903" s="719" t="inlineStr">
+        <is>
+          <t>Senior Paid Media Strategist</t>
+        </is>
+      </c>
+      <c r="E903" s="722" t="n">
+        <v>31</v>
+      </c>
+      <c r="F903" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G903" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H903" s="719" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I903" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J903" s="719" t="n"/>
+      <c r="K903" s="719" t="inlineStr">
+        <is>
+          <t>$100 per hour</t>
+        </is>
+      </c>
+      <c r="L903" s="720" t="n">
+        <v>46283</v>
+      </c>
+      <c r="M903" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N903" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O903" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P903" s="719" t="n"/>
+      <c r="Q903" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/2611974851401550447?p=1&amp;pos=16&amp;rgn=55157&amp;cid=19881&amp;ckey=Senior+Paid+Search+Strategist&amp;jobAge=115&amp;brelb=10&amp;scr=3589.1536&amp;bscr=3589.1536&amp;aq=-427099300053651923&amp;elckey=5303113098520002782</t>
+        </is>
+      </c>
+      <c r="R903" s="719" t="n"/>
+      <c r="S903" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T903" s="719" t="n"/>
+      <c r="U903" s="719" t="n"/>
+      <c r="V903" s="719" t="n"/>
+      <c r="W903" s="719" t="n"/>
+    </row>
+    <row r="904">
+      <c r="A904" s="719" t="n">
+        <v>903</v>
+      </c>
+      <c r="B904" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C904" s="719" t="inlineStr">
+        <is>
+          <t>Regex SEO</t>
+        </is>
+      </c>
+      <c r="D904" s="719" t="inlineStr">
+        <is>
+          <t>Senior Paid Media Strategist (PPC | Home Services)</t>
+        </is>
+      </c>
+      <c r="E904" s="722" t="n">
+        <v>43</v>
+      </c>
+      <c r="F904" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G904" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H904" s="719" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="I904" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J904" s="719" t="n"/>
+      <c r="K904" s="719" t="inlineStr">
+        <is>
+          <t>$4,000 - $8,000 per month</t>
+        </is>
+      </c>
+      <c r="L904" s="720" t="n">
+        <v>46283</v>
+      </c>
+      <c r="M904" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N904" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O904" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P904" s="719" t="n"/>
+      <c r="Q904" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-8055074814535542540?p=1&amp;pos=18&amp;rgn=55157&amp;cid=19881&amp;ckey=Senior+Paid+Search+Strategist&amp;jobAge=115&amp;brelb=100&amp;scr=3113.3591&amp;bscr=3113.3591&amp;aq=-427099300053651923&amp;elckey=5303113098520002782</t>
+        </is>
+      </c>
+      <c r="R904" s="719" t="n"/>
+      <c r="S904" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T904" s="719" t="n"/>
+      <c r="U904" s="719" t="n"/>
+      <c r="V904" s="719" t="n"/>
+      <c r="W904" s="719" t="n"/>
+    </row>
+    <row r="905">
+      <c r="A905" s="719" t="n">
+        <v>904</v>
+      </c>
+      <c r="B905" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C905" s="719" t="inlineStr">
+        <is>
+          <t>24 Seven Talent</t>
+        </is>
+      </c>
+      <c r="D905" s="719" t="inlineStr">
+        <is>
+          <t>Senior Paid Media Strategist</t>
+        </is>
+      </c>
+      <c r="E905" s="722" t="n">
+        <v>35</v>
+      </c>
+      <c r="F905" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G905" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H905" s="719" t="inlineStr">
+        <is>
+          <t>California, MO</t>
+        </is>
+      </c>
+      <c r="I905" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J905" s="719" t="n"/>
+      <c r="K905" s="719" t="n"/>
+      <c r="L905" s="720" t="n">
+        <v>46282</v>
+      </c>
+      <c r="M905" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N905" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O905" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P905" s="719" t="n"/>
+      <c r="Q905" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/1512123861419150239?p=1&amp;pos=19&amp;rgn=55157&amp;cid=19881&amp;ckey=Senior+Paid+Search+Strategist&amp;jobAge=139&amp;brelb=100&amp;scr=3096.0674&amp;bscr=3096.0674&amp;aq=-427099300053651923&amp;elckey=5303113098520002782</t>
+        </is>
+      </c>
+      <c r="R905" s="719" t="n"/>
+      <c r="S905" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T905" s="719" t="n"/>
+      <c r="U905" s="719" t="n"/>
+      <c r="V905" s="719" t="n"/>
+      <c r="W905" s="719" t="n"/>
+    </row>
+    <row r="906">
+      <c r="A906" s="719" t="n">
+        <v>905</v>
+      </c>
+      <c r="B906" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C906" s="719" t="inlineStr">
+        <is>
+          <t>321 the Agency</t>
+        </is>
+      </c>
+      <c r="D906" s="719" t="inlineStr">
+        <is>
+          <t>Director of Digital Marketing</t>
+        </is>
+      </c>
+      <c r="E906" s="722" t="n">
+        <v>55</v>
+      </c>
+      <c r="F906" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G906" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H906" s="719" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I906" s="719" t="inlineStr">
+        <is>
+          <t>remote</t>
+        </is>
+      </c>
+      <c r="J906" s="719" t="n"/>
+      <c r="K906" s="719" t="inlineStr">
+        <is>
+          <t>$100k - $115k</t>
+        </is>
+      </c>
+      <c r="L906" s="720" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M906" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N906" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O906" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P906" s="719" t="n"/>
+      <c r="Q906" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/8412425693059398420?p=1&amp;pos=3&amp;rgn=55157&amp;cid=19881&amp;ckey=Director+of+Digital+Marketing&amp;jobAge=43&amp;brelb=10&amp;scr=184.89296&amp;bscr=184.89296&amp;aq=462242672333371932&amp;elckey=-1717610386031322039</t>
+        </is>
+      </c>
+      <c r="R906" s="719" t="n"/>
+      <c r="S906" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T906" s="719" t="n"/>
+      <c r="U906" s="719" t="n"/>
+      <c r="V906" s="719" t="n"/>
+      <c r="W906" s="719" t="n"/>
+    </row>
+    <row r="907">
+      <c r="A907" s="719" t="n">
+        <v>906</v>
+      </c>
+      <c r="B907" s="719" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="C907" s="719" t="inlineStr">
+        <is>
+          <t>Unity Technologies</t>
+        </is>
+      </c>
+      <c r="D907" s="719" t="inlineStr">
+        <is>
+          <t>Senior Performance Marketing Manager - SEM</t>
+        </is>
+      </c>
+      <c r="E907" s="722" t="n">
+        <v>66</v>
+      </c>
+      <c r="F907" s="723" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G907" s="719" t="inlineStr">
+        <is>
+          <t>Below Threshold</t>
+        </is>
+      </c>
+      <c r="H907" s="719" t="inlineStr">
+        <is>
+          <t>Florida</t>
+        </is>
+      </c>
+      <c r="I907" s="719" t="inlineStr">
+        <is>
+          <t>on-site</t>
+        </is>
+      </c>
+      <c r="J907" s="719" t="n"/>
+      <c r="K907" s="719" t="inlineStr">
+        <is>
+          <t>$87.4k - $131.2k</t>
+        </is>
+      </c>
+      <c r="L907" s="720" t="n">
+        <v>46285</v>
+      </c>
+      <c r="M907" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="N907" s="720" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O907" s="719" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="P907" s="719" t="n"/>
+      <c r="Q907" s="1" t="inlineStr">
+        <is>
+          <t>https://jooble.org/away/-601130303526563547?p=1&amp;pos=10&amp;rgn=55157&amp;cid=19881&amp;ckey=Director+of+Performance+Marketing&amp;jobAge=63&amp;brelb=100&amp;scr=105.12633&amp;bscr=105.12633&amp;aq=-7205443806904435238&amp;elckey=4704404259572399187</t>
+        </is>
+      </c>
+      <c r="R907" s="719" t="n"/>
+      <c r="S907" s="719" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="T907" s="719" t="n"/>
+      <c r="U907" s="719" t="n"/>
+      <c r="V907" s="719" t="n"/>
+      <c r="W907" s="719" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W848"/>
+  <autoFilter ref="A1:W907"/>
   <conditionalFormatting sqref="A2:W848">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>$G2="Confirmed Strong Match"</formula>
@@ -69735,6 +74178,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q846" r:id="rId889"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q847" r:id="rId890"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q848" r:id="rId891"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q849" r:id="rId892"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q850" r:id="rId893"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q851" r:id="rId894"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q852" r:id="rId895"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q853" r:id="rId896"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q854" r:id="rId897"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q855" r:id="rId898"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q856" r:id="rId899"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q857" r:id="rId900"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q858" r:id="rId901"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q859" r:id="rId902"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q860" r:id="rId903"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q861" r:id="rId904"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q862" r:id="rId905"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q863" r:id="rId906"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q864" r:id="rId907"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q865" r:id="rId908"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q866" r:id="rId909"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q867" r:id="rId910"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q868" r:id="rId911"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q869" r:id="rId912"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q870" r:id="rId913"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q871" r:id="rId914"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q872" r:id="rId915"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q873" r:id="rId916"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q874" r:id="rId917"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q875" r:id="rId918"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q876" r:id="rId919"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q877" r:id="rId920"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q878" r:id="rId921"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q879" r:id="rId922"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q880" r:id="rId923"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q881" r:id="rId924"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q882" r:id="rId925"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q883" r:id="rId926"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q884" r:id="rId927"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q885" r:id="rId928"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q886" r:id="rId929"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q887" r:id="rId930"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q888" r:id="rId931"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q889" r:id="rId932"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V889" r:id="rId933"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q890" r:id="rId934"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q891" r:id="rId935"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q892" r:id="rId936"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q893" r:id="rId937"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q894" r:id="rId938"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q895" r:id="rId939"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q896" r:id="rId940"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q897" r:id="rId941"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q898" r:id="rId942"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q899" r:id="rId943"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q900" r:id="rId944"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q901" r:id="rId945"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q902" r:id="rId946"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q903" r:id="rId947"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q904" r:id="rId948"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q905" r:id="rId949"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q906" r:id="rId950"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q907" r:id="rId951"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>